<commit_message>
pushing latest changes for deprivation model baseline
</commit_message>
<xml_diff>
--- a/src/index_travel_accessibility/data/processed/calculated_metrics_from_travel_time.xlsx
+++ b/src/index_travel_accessibility/data/processed/calculated_metrics_from_travel_time.xlsx
@@ -472,19 +472,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17.468</v>
+        <v>17.812</v>
       </c>
       <c r="C2" t="n">
-        <v>12.08</v>
+        <v>12.66</v>
       </c>
       <c r="D2" t="n">
-        <v>28.85</v>
+        <v>29.056</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7685386286068879</v>
+        <v>0.8220155038759691</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2511848341232228</v>
+        <v>0.3061611374407583</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -506,7 +506,7 @@
         <v>20.328</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5507291343468818</v>
+        <v>0.5510077519379845</v>
       </c>
       <c r="F3" t="n">
         <v>0.7611374407582939</v>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12.514</v>
+        <v>12.51</v>
       </c>
       <c r="C4" t="n">
         <v>9.43</v>
@@ -537,7 +537,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4064773527340999</v>
+        <v>0.3968835930339138</v>
       </c>
     </row>
     <row r="5">
@@ -556,13 +556,13 @@
         <v>27.038</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7105181507911884</v>
+        <v>0.7106976744186048</v>
       </c>
       <c r="F5" t="n">
         <v>0.5924170616113744</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7873738559023705</v>
+        <v>0.7687901008249315</v>
       </c>
     </row>
     <row r="6">
@@ -587,7 +587,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5817883126026757</v>
+        <v>0.5680568285976172</v>
       </c>
     </row>
     <row r="7">
@@ -606,13 +606,13 @@
         <v>24.446</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9959664908470369</v>
+        <v>0.995968992248062</v>
       </c>
       <c r="F7" t="n">
         <v>0.78957345971564</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4832199014315892</v>
+        <v>0.4718148487626035</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added results for this branch for evaluation for two hospital prediction
</commit_message>
<xml_diff>
--- a/src/index_travel_accessibility/data/processed/calculated_metrics_from_travel_time.xlsx
+++ b/src/index_travel_accessibility/data/processed/calculated_metrics_from_travel_time.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17.466</v>
+        <v>17.468</v>
       </c>
       <c r="C2" t="n">
         <v>12.08</v>
@@ -481,10 +481,10 @@
         <v>28.85</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7771070168561351</v>
+        <v>0.7686821705426355</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2423411065386374</v>
+        <v>0.2511848341232228</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16.022</v>
+        <v>16.064</v>
       </c>
       <c r="C3" t="n">
         <v>17.46</v>
@@ -506,10 +506,10 @@
         <v>20.328</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5506860054880437</v>
+        <v>0.5510077519379845</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7343392775491541</v>
+        <v>0.7611374407582939</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -547,22 +547,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18.6025</v>
+        <v>17.094</v>
       </c>
       <c r="C5" t="n">
-        <v>20.035</v>
+        <v>15.68</v>
       </c>
       <c r="D5" t="n">
-        <v>27.2035</v>
+        <v>27.038</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9553116424931399</v>
+        <v>0.7106976744186048</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9698216735253771</v>
+        <v>0.5924170616113744</v>
       </c>
       <c r="G5" t="n">
-        <v>0.806794179770007</v>
+        <v>0.7873738559023705</v>
       </c>
     </row>
     <row r="6">
@@ -572,13 +572,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18.8875</v>
+        <v>18.96</v>
       </c>
       <c r="C6" t="n">
-        <v>20.365</v>
+        <v>19.98</v>
       </c>
       <c r="D6" t="n">
-        <v>25.5695</v>
+        <v>25.286</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -587,7 +587,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6150551513729171</v>
+        <v>0.5817883126026757</v>
       </c>
     </row>
     <row r="7">
@@ -597,22 +597,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18.87333333333333</v>
+        <v>18.934</v>
       </c>
       <c r="C7" t="n">
         <v>17.76</v>
       </c>
       <c r="D7" t="n">
-        <v>23.079</v>
+        <v>24.446</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9977786488958582</v>
+        <v>0.995968992248062</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7617741197988112</v>
+        <v>0.78957345971564</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3228115465853088</v>
+        <v>0.4832199014315892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>